<commit_message>
Save a restore point before the shared BonsaiCore domain move.
This snapshot captures the working Mac product, docs, and the current iOS demo so we can return here if the canonical-domain change needs to be undone.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bonsai Hub/Resources/Import/Bonsai Database Olaf Barmen 3.xlsx
+++ b/Bonsai Hub/Resources/Import/Bonsai Database Olaf Barmen 3.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10710"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/olafbarmen/Developer/Falo Universe/Bonsai Hub/Bonsai Hub/Resources/Import/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olaf\iCloudDrive\Documents\Bonsai\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{501626A4-3C99-584C-8DC1-26B847AD995F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADC0AB16-E9CA-44B2-89B5-E68FF9FD5D29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="20580" windowHeight="22480" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43125" yWindow="0" windowWidth="33510" windowHeight="11205" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -2638,7 +2638,6 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -2674,7 +2673,6 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="8">
@@ -3137,93 +3135,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="180"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3242,17 +3161,14 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -3263,10 +3179,92 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3771,10 +3769,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Ark1"/>
   <dimension ref="A1:B1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.33203125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="14.390625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="46.33203125" customWidth="1"/>
-    <col min="3" max="26" width="9.33203125" customWidth="1"/>
+    <col min="1" max="2" width="46.2734375" customWidth="1"/>
+    <col min="3" max="26" width="9.28125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -5110,30 +5108,30 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Ark3"/>
   <dimension ref="A1:AD999"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.33203125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="14.390625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="11.5" customWidth="1"/>
-    <col min="3" max="5" width="20.6640625" customWidth="1"/>
-    <col min="6" max="6" width="27.6640625" customWidth="1"/>
-    <col min="7" max="7" width="50.6640625" customWidth="1"/>
-    <col min="8" max="8" width="17" customWidth="1"/>
-    <col min="9" max="9" width="20.6640625" style="15" customWidth="1"/>
-    <col min="10" max="13" width="20.6640625" customWidth="1"/>
-    <col min="14" max="14" width="16.33203125" customWidth="1"/>
-    <col min="15" max="15" width="8.6640625" customWidth="1"/>
-    <col min="16" max="16" width="15" customWidth="1"/>
-    <col min="17" max="17" width="17" customWidth="1"/>
-    <col min="18" max="18" width="15" customWidth="1"/>
-    <col min="19" max="25" width="20.6640625" customWidth="1"/>
-    <col min="26" max="26" width="20.6640625" style="15" customWidth="1"/>
-    <col min="27" max="27" width="20.6640625" customWidth="1"/>
-    <col min="28" max="28" width="20.6640625" style="15" customWidth="1"/>
-    <col min="29" max="29" width="7.33203125" customWidth="1"/>
-    <col min="30" max="30" width="50.1640625" customWidth="1"/>
+    <col min="1" max="1" width="24.078125" customWidth="1"/>
+    <col min="2" max="2" width="11.43359375" customWidth="1"/>
+    <col min="3" max="5" width="20.71484375" customWidth="1"/>
+    <col min="6" max="6" width="27.7109375" customWidth="1"/>
+    <col min="7" max="7" width="50.71484375" customWidth="1"/>
+    <col min="8" max="8" width="16.94921875" customWidth="1"/>
+    <col min="9" max="9" width="20.71484375" style="15" customWidth="1"/>
+    <col min="10" max="13" width="20.71484375" customWidth="1"/>
+    <col min="14" max="14" width="16.41015625" customWidth="1"/>
+    <col min="15" max="15" width="8.7421875" customWidth="1"/>
+    <col min="16" max="16" width="14.9296875" customWidth="1"/>
+    <col min="17" max="17" width="17.08203125" customWidth="1"/>
+    <col min="18" max="18" width="14.9296875" customWidth="1"/>
+    <col min="19" max="25" width="20.71484375" customWidth="1"/>
+    <col min="26" max="26" width="20.71484375" style="15" customWidth="1"/>
+    <col min="27" max="27" width="20.71484375" customWidth="1"/>
+    <col min="28" max="28" width="20.71484375" style="15" customWidth="1"/>
+    <col min="29" max="29" width="7.26171875" customWidth="1"/>
+    <col min="30" max="30" width="50.17578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
         <v>53</v>
       </c>
@@ -48168,10 +48166,10 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58DFFF9B-5B05-4458-BA98-167A42F0BE98}">
   <dimension ref="B2:S52"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.76171875" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="7" max="7" width="5.1640625" customWidth="1"/>
+    <col min="2" max="2" width="14.9296875" customWidth="1"/>
+    <col min="7" max="7" width="5.24609375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:19" x14ac:dyDescent="0.2">
@@ -49177,54 +49175,54 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Ark4"/>
   <dimension ref="A1:BD1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.33203125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="14.390625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.33203125" customWidth="1"/>
-    <col min="2" max="2" width="9.33203125" customWidth="1"/>
-    <col min="3" max="3" width="13.5" customWidth="1"/>
-    <col min="4" max="4" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.2578125" customWidth="1"/>
+    <col min="2" max="2" width="9.28125" customWidth="1"/>
+    <col min="3" max="3" width="13.44921875" customWidth="1"/>
+    <col min="4" max="4" width="18.16015625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.97265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="10.22265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.9140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.33203125" customWidth="1"/>
-    <col min="14" max="14" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.5" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="8.5" customWidth="1"/>
-    <col min="17" max="17" width="21.1640625" customWidth="1"/>
-    <col min="18" max="18" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="26" max="27" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="15.1640625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="17.83203125" bestFit="1" customWidth="1"/>
-    <col min="32" max="34" width="13" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="15.1640625" bestFit="1" customWidth="1"/>
-    <col min="36" max="38" width="8.5" customWidth="1"/>
-    <col min="39" max="39" width="16.33203125" customWidth="1"/>
-    <col min="40" max="40" width="5.1640625" customWidth="1"/>
-    <col min="41" max="41" width="15.6640625" customWidth="1"/>
-    <col min="42" max="42" width="9.33203125" customWidth="1"/>
-    <col min="43" max="43" width="13.5" customWidth="1"/>
-    <col min="44" max="44" width="9.33203125" customWidth="1"/>
-    <col min="45" max="45" width="10.83203125" customWidth="1"/>
-    <col min="46" max="46" width="9.33203125" customWidth="1"/>
-    <col min="47" max="47" width="10.83203125" customWidth="1"/>
-    <col min="48" max="48" width="9.33203125" customWidth="1"/>
+    <col min="11" max="11" width="10.22265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.4140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.4140625" customWidth="1"/>
+    <col min="14" max="14" width="8.7421875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.47265625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.47265625" customWidth="1"/>
+    <col min="17" max="17" width="21.1171875" customWidth="1"/>
+    <col min="18" max="18" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.22265625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="15.73828125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.0078125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.71875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="14.66015625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="14.125" bestFit="1" customWidth="1"/>
+    <col min="26" max="27" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="15.19921875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="19.37109375" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="13.44921875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="17.890625" bestFit="1" customWidth="1"/>
+    <col min="32" max="34" width="13.046875" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="15.19921875" bestFit="1" customWidth="1"/>
+    <col min="36" max="38" width="8.47265625" customWidth="1"/>
+    <col min="39" max="39" width="16.27734375" customWidth="1"/>
+    <col min="40" max="40" width="5.24609375" customWidth="1"/>
+    <col min="41" max="41" width="15.73828125" customWidth="1"/>
+    <col min="42" max="42" width="9.28125" customWidth="1"/>
+    <col min="43" max="43" width="13.44921875" customWidth="1"/>
+    <col min="44" max="44" width="9.28125" customWidth="1"/>
+    <col min="45" max="45" width="10.89453125" customWidth="1"/>
+    <col min="46" max="46" width="9.28125" customWidth="1"/>
+    <col min="47" max="47" width="10.89453125" customWidth="1"/>
+    <col min="48" max="48" width="9.28125" customWidth="1"/>
     <col min="49" max="49" width="18.83203125" customWidth="1"/>
-    <col min="50" max="53" width="9.33203125" customWidth="1"/>
-    <col min="54" max="54" width="53.33203125" customWidth="1"/>
-    <col min="55" max="56" width="9.33203125" customWidth="1"/>
+    <col min="50" max="53" width="9.28125" customWidth="1"/>
+    <col min="54" max="54" width="53.26953125" customWidth="1"/>
+    <col min="55" max="56" width="9.28125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:56" x14ac:dyDescent="0.2">
@@ -49465,7 +49463,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="4" spans="1:56" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A4" s="25" t="s">
         <v>218</v>
       </c>
@@ -51959,7 +51957,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA64F3A-8B61-6A43-B279-B4B0B3711DD4}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.28125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -51971,36 +51969,36 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="B1:Y114"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.33203125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="14.390625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.6640625" customWidth="1"/>
-    <col min="2" max="2" width="10.1640625" style="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13" style="24" customWidth="1"/>
-    <col min="4" max="4" width="13.6640625" style="24" customWidth="1"/>
-    <col min="5" max="5" width="13" style="80" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.1640625" customWidth="1"/>
-    <col min="8" max="8" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.83203125" customWidth="1"/>
-    <col min="11" max="11" width="13" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.1640625" customWidth="1"/>
-    <col min="13" max="13" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.1640625" customWidth="1"/>
-    <col min="18" max="18" width="4.83203125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.703125" customWidth="1"/>
+    <col min="2" max="2" width="10.22265625" style="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.046875" style="24" customWidth="1"/>
+    <col min="4" max="4" width="13.5859375" style="24" customWidth="1"/>
+    <col min="5" max="5" width="13.046875" style="80" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.046875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.22265625" customWidth="1"/>
+    <col min="8" max="8" width="15.46875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.28125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.890625" customWidth="1"/>
+    <col min="11" max="11" width="13.046875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.22265625" customWidth="1"/>
+    <col min="13" max="13" width="7.26171875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.22265625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.22265625" customWidth="1"/>
+    <col min="18" max="18" width="4.83984375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.28125" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.1640625" customWidth="1"/>
-    <col min="23" max="23" width="4.83203125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.22265625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.22265625" customWidth="1"/>
+    <col min="23" max="23" width="4.83984375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="9.28125" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="11.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:25" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B1" s="23"/>
       <c r="C1" s="23"/>
       <c r="D1" s="23"/>
@@ -52015,74 +52013,74 @@
       <c r="M1" s="5"/>
       <c r="N1" s="5"/>
     </row>
-    <row r="2" spans="2:25" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="140" t="s">
+    <row r="2" spans="2:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="172" t="s">
         <v>45</v>
       </c>
-      <c r="C2" s="141"/>
-      <c r="D2" s="141"/>
-      <c r="E2" s="142"/>
-      <c r="F2" s="142"/>
-      <c r="G2" s="142"/>
-      <c r="H2" s="142"/>
-      <c r="I2" s="142"/>
-      <c r="J2" s="142"/>
-      <c r="K2" s="142"/>
-      <c r="L2" s="142"/>
-      <c r="M2" s="142"/>
-      <c r="N2" s="142"/>
-      <c r="O2" s="142"/>
-      <c r="P2" s="142"/>
-      <c r="Q2" s="142"/>
-      <c r="R2" s="142"/>
-      <c r="S2" s="142"/>
-      <c r="T2" s="142"/>
-      <c r="U2" s="142"/>
-      <c r="V2" s="142"/>
-      <c r="W2" s="142"/>
-      <c r="X2" s="142"/>
-      <c r="Y2" s="143"/>
-    </row>
-    <row r="3" spans="2:25" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="147" t="s">
+      <c r="C2" s="173"/>
+      <c r="D2" s="173"/>
+      <c r="E2" s="174"/>
+      <c r="F2" s="174"/>
+      <c r="G2" s="174"/>
+      <c r="H2" s="174"/>
+      <c r="I2" s="174"/>
+      <c r="J2" s="174"/>
+      <c r="K2" s="174"/>
+      <c r="L2" s="174"/>
+      <c r="M2" s="174"/>
+      <c r="N2" s="174"/>
+      <c r="O2" s="174"/>
+      <c r="P2" s="174"/>
+      <c r="Q2" s="174"/>
+      <c r="R2" s="174"/>
+      <c r="S2" s="174"/>
+      <c r="T2" s="174"/>
+      <c r="U2" s="174"/>
+      <c r="V2" s="174"/>
+      <c r="W2" s="174"/>
+      <c r="X2" s="174"/>
+      <c r="Y2" s="175"/>
+    </row>
+    <row r="3" spans="2:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="155" t="s">
         <v>722</v>
       </c>
-      <c r="C3" s="144" t="s">
+      <c r="C3" s="163" t="s">
         <v>720</v>
       </c>
-      <c r="D3" s="144" t="s">
+      <c r="D3" s="163" t="s">
         <v>724</v>
       </c>
       <c r="E3" s="81"/>
-      <c r="F3" s="132" t="s">
+      <c r="F3" s="165" t="s">
         <v>559</v>
       </c>
-      <c r="G3" s="132"/>
-      <c r="H3" s="133"/>
-      <c r="I3" s="133"/>
-      <c r="J3" s="134"/>
-      <c r="K3" s="131" t="s">
+      <c r="G3" s="165"/>
+      <c r="H3" s="166"/>
+      <c r="I3" s="166"/>
+      <c r="J3" s="167"/>
+      <c r="K3" s="169" t="s">
         <v>560</v>
       </c>
-      <c r="L3" s="132"/>
-      <c r="M3" s="133"/>
-      <c r="N3" s="133"/>
-      <c r="O3" s="134"/>
-      <c r="P3" s="131"/>
-      <c r="Q3" s="132"/>
-      <c r="R3" s="133"/>
-      <c r="S3" s="133"/>
-      <c r="T3" s="134"/>
-      <c r="U3" s="135"/>
-      <c r="V3" s="136"/>
-      <c r="W3" s="133"/>
-      <c r="X3" s="133"/>
-      <c r="Y3" s="134"/>
+      <c r="L3" s="165"/>
+      <c r="M3" s="166"/>
+      <c r="N3" s="166"/>
+      <c r="O3" s="167"/>
+      <c r="P3" s="169"/>
+      <c r="Q3" s="165"/>
+      <c r="R3" s="166"/>
+      <c r="S3" s="166"/>
+      <c r="T3" s="167"/>
+      <c r="U3" s="170"/>
+      <c r="V3" s="171"/>
+      <c r="W3" s="166"/>
+      <c r="X3" s="166"/>
+      <c r="Y3" s="167"/>
     </row>
     <row r="4" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B4" s="148"/>
-      <c r="C4" s="145"/>
-      <c r="D4" s="145"/>
+      <c r="B4" s="156"/>
+      <c r="C4" s="151"/>
+      <c r="D4" s="151"/>
       <c r="E4" s="82"/>
       <c r="F4" s="64" t="s">
         <v>46</v>
@@ -52146,9 +52144,9 @@
       </c>
     </row>
     <row r="5" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B5" s="148"/>
-      <c r="C5" s="145"/>
-      <c r="D5" s="145"/>
+      <c r="B5" s="156"/>
+      <c r="C5" s="151"/>
+      <c r="D5" s="151"/>
       <c r="E5" s="85" t="s">
         <v>726</v>
       </c>
@@ -52174,9 +52172,9 @@
       <c r="Y5" s="29"/>
     </row>
     <row r="6" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B6" s="148"/>
-      <c r="C6" s="145"/>
-      <c r="D6" s="145"/>
+      <c r="B6" s="156"/>
+      <c r="C6" s="151"/>
+      <c r="D6" s="151"/>
       <c r="E6" s="127" t="s">
         <v>742</v>
       </c>
@@ -52202,9 +52200,9 @@
       <c r="Y6" s="29"/>
     </row>
     <row r="7" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B7" s="148"/>
-      <c r="C7" s="145"/>
-      <c r="D7" s="145"/>
+      <c r="B7" s="156"/>
+      <c r="C7" s="151"/>
+      <c r="D7" s="151"/>
       <c r="E7" s="127" t="s">
         <v>743</v>
       </c>
@@ -52230,9 +52228,9 @@
       <c r="Y7" s="29"/>
     </row>
     <row r="8" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B8" s="148"/>
-      <c r="C8" s="145"/>
-      <c r="D8" s="145"/>
+      <c r="B8" s="156"/>
+      <c r="C8" s="151"/>
+      <c r="D8" s="151"/>
       <c r="E8" s="127" t="s">
         <v>744</v>
       </c>
@@ -52258,9 +52256,9 @@
       <c r="Y8" s="29"/>
     </row>
     <row r="9" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B9" s="148"/>
-      <c r="C9" s="145"/>
-      <c r="D9" s="145"/>
+      <c r="B9" s="156"/>
+      <c r="C9" s="151"/>
+      <c r="D9" s="151"/>
       <c r="E9" s="127" t="s">
         <v>745</v>
       </c>
@@ -52285,9 +52283,9 @@
       <c r="Y9" s="29"/>
     </row>
     <row r="10" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="148"/>
-      <c r="C10" s="145"/>
-      <c r="D10" s="145"/>
+      <c r="B10" s="156"/>
+      <c r="C10" s="151"/>
+      <c r="D10" s="151"/>
       <c r="E10" s="127" t="s">
         <v>746</v>
       </c>
@@ -52312,9 +52310,9 @@
       <c r="Y10" s="29"/>
     </row>
     <row r="11" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B11" s="148"/>
-      <c r="C11" s="145"/>
-      <c r="D11" s="145"/>
+      <c r="B11" s="156"/>
+      <c r="C11" s="151"/>
+      <c r="D11" s="151"/>
       <c r="E11" s="71"/>
       <c r="F11" s="66"/>
       <c r="G11" s="66"/>
@@ -52328,9 +52326,9 @@
       <c r="Y11" s="29"/>
     </row>
     <row r="12" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="148"/>
-      <c r="C12" s="146"/>
-      <c r="D12" s="146"/>
+      <c r="B12" s="156"/>
+      <c r="C12" s="162"/>
+      <c r="D12" s="162"/>
       <c r="E12" s="83"/>
       <c r="F12" s="31"/>
       <c r="G12" s="31"/>
@@ -52353,44 +52351,44 @@
       <c r="X12" s="31"/>
       <c r="Y12" s="32"/>
     </row>
-    <row r="13" spans="2:25" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="148"/>
-      <c r="C13" s="144" t="s">
+    <row r="13" spans="2:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="156"/>
+      <c r="C13" s="163" t="s">
         <v>719</v>
       </c>
-      <c r="D13" s="144" t="s">
+      <c r="D13" s="163" t="s">
         <v>725</v>
       </c>
       <c r="E13" s="75"/>
-      <c r="F13" s="131" t="s">
+      <c r="F13" s="169" t="s">
         <v>562</v>
       </c>
-      <c r="G13" s="132"/>
-      <c r="H13" s="133"/>
-      <c r="I13" s="133"/>
-      <c r="J13" s="134"/>
-      <c r="K13" s="135" t="s">
+      <c r="G13" s="165"/>
+      <c r="H13" s="166"/>
+      <c r="I13" s="166"/>
+      <c r="J13" s="167"/>
+      <c r="K13" s="170" t="s">
         <v>564</v>
       </c>
-      <c r="L13" s="136"/>
-      <c r="M13" s="133"/>
-      <c r="N13" s="133"/>
-      <c r="O13" s="134"/>
-      <c r="P13" s="131"/>
-      <c r="Q13" s="132"/>
-      <c r="R13" s="133"/>
-      <c r="S13" s="133"/>
-      <c r="T13" s="134"/>
-      <c r="U13" s="135"/>
-      <c r="V13" s="136"/>
-      <c r="W13" s="133"/>
-      <c r="X13" s="133"/>
-      <c r="Y13" s="134"/>
+      <c r="L13" s="171"/>
+      <c r="M13" s="166"/>
+      <c r="N13" s="166"/>
+      <c r="O13" s="167"/>
+      <c r="P13" s="169"/>
+      <c r="Q13" s="165"/>
+      <c r="R13" s="166"/>
+      <c r="S13" s="166"/>
+      <c r="T13" s="167"/>
+      <c r="U13" s="170"/>
+      <c r="V13" s="171"/>
+      <c r="W13" s="166"/>
+      <c r="X13" s="166"/>
+      <c r="Y13" s="167"/>
     </row>
     <row r="14" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B14" s="148"/>
-      <c r="C14" s="145"/>
-      <c r="D14" s="145"/>
+      <c r="B14" s="156"/>
+      <c r="C14" s="151"/>
+      <c r="D14" s="151"/>
       <c r="E14" s="76"/>
       <c r="F14" s="26" t="s">
         <v>46</v>
@@ -52454,9 +52452,9 @@
       </c>
     </row>
     <row r="15" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B15" s="148"/>
-      <c r="C15" s="145"/>
-      <c r="D15" s="145"/>
+      <c r="B15" s="156"/>
+      <c r="C15" s="151"/>
+      <c r="D15" s="151"/>
       <c r="E15" s="130" t="s">
         <v>747</v>
       </c>
@@ -52483,9 +52481,9 @@
       <c r="Y15" s="29"/>
     </row>
     <row r="16" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B16" s="148"/>
-      <c r="C16" s="145"/>
-      <c r="D16" s="145"/>
+      <c r="B16" s="156"/>
+      <c r="C16" s="151"/>
+      <c r="D16" s="151"/>
       <c r="E16" s="130" t="s">
         <v>748</v>
       </c>
@@ -52512,10 +52510,10 @@
       <c r="Y16" s="29"/>
     </row>
     <row r="17" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B17" s="148"/>
-      <c r="C17" s="145"/>
-      <c r="D17" s="145"/>
-      <c r="E17" s="171" t="s">
+      <c r="B17" s="156"/>
+      <c r="C17" s="151"/>
+      <c r="D17" s="151"/>
+      <c r="E17" s="150" t="s">
         <v>756</v>
       </c>
       <c r="F17" s="129" t="s">
@@ -52552,10 +52550,10 @@
       <c r="Y17" s="29"/>
     </row>
     <row r="18" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B18" s="148"/>
-      <c r="C18" s="145"/>
-      <c r="D18" s="145"/>
-      <c r="E18" s="145"/>
+      <c r="B18" s="156"/>
+      <c r="C18" s="151"/>
+      <c r="D18" s="151"/>
+      <c r="E18" s="151"/>
       <c r="F18" s="28"/>
       <c r="J18" s="29"/>
       <c r="K18" s="129" t="s">
@@ -52578,11 +52576,11 @@
       <c r="U18" s="28"/>
       <c r="Y18" s="29"/>
     </row>
-    <row r="19" spans="2:25" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="148"/>
-      <c r="C19" s="145"/>
-      <c r="D19" s="145"/>
-      <c r="E19" s="145"/>
+    <row r="19" spans="2:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="156"/>
+      <c r="C19" s="151"/>
+      <c r="D19" s="151"/>
+      <c r="E19" s="151"/>
       <c r="F19" s="28"/>
       <c r="J19" s="29"/>
       <c r="K19" s="68" t="s">
@@ -52605,42 +52603,42 @@
       <c r="U19" s="28"/>
       <c r="Y19" s="29"/>
     </row>
-    <row r="20" spans="2:25" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="148"/>
-      <c r="C20" s="144" t="s">
+    <row r="20" spans="2:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="156"/>
+      <c r="C20" s="163" t="s">
         <v>721</v>
       </c>
-      <c r="D20" s="173" t="s">
+      <c r="D20" s="161" t="s">
         <v>725</v>
       </c>
       <c r="E20" s="75"/>
-      <c r="F20" s="137" t="s">
+      <c r="F20" s="168" t="s">
         <v>728</v>
       </c>
-      <c r="G20" s="132"/>
-      <c r="H20" s="132"/>
-      <c r="I20" s="132"/>
-      <c r="J20" s="138"/>
-      <c r="K20" s="135"/>
-      <c r="L20" s="136"/>
-      <c r="M20" s="136"/>
-      <c r="N20" s="136"/>
-      <c r="O20" s="139"/>
-      <c r="P20" s="131"/>
-      <c r="Q20" s="132"/>
-      <c r="R20" s="132"/>
-      <c r="S20" s="132"/>
-      <c r="T20" s="138"/>
-      <c r="U20" s="135"/>
-      <c r="V20" s="136"/>
-      <c r="W20" s="136"/>
-      <c r="X20" s="136"/>
-      <c r="Y20" s="139"/>
+      <c r="G20" s="165"/>
+      <c r="H20" s="165"/>
+      <c r="I20" s="165"/>
+      <c r="J20" s="177"/>
+      <c r="K20" s="170"/>
+      <c r="L20" s="171"/>
+      <c r="M20" s="171"/>
+      <c r="N20" s="171"/>
+      <c r="O20" s="178"/>
+      <c r="P20" s="169"/>
+      <c r="Q20" s="165"/>
+      <c r="R20" s="165"/>
+      <c r="S20" s="165"/>
+      <c r="T20" s="177"/>
+      <c r="U20" s="170"/>
+      <c r="V20" s="171"/>
+      <c r="W20" s="171"/>
+      <c r="X20" s="171"/>
+      <c r="Y20" s="178"/>
     </row>
     <row r="21" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="148"/>
-      <c r="C21" s="145"/>
-      <c r="D21" s="145"/>
+      <c r="B21" s="156"/>
+      <c r="C21" s="151"/>
+      <c r="D21" s="151"/>
       <c r="E21" s="76"/>
       <c r="F21" s="26" t="s">
         <v>46</v>
@@ -52704,9 +52702,9 @@
       </c>
     </row>
     <row r="22" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="148"/>
-      <c r="C22" s="145"/>
-      <c r="D22" s="145"/>
+      <c r="B22" s="156"/>
+      <c r="C22" s="151"/>
+      <c r="D22" s="151"/>
       <c r="E22" s="130" t="s">
         <v>757</v>
       </c>
@@ -52728,9 +52726,9 @@
       <c r="Y22" s="29"/>
     </row>
     <row r="23" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="148"/>
-      <c r="C23" s="145"/>
-      <c r="D23" s="145"/>
+      <c r="B23" s="156"/>
+      <c r="C23" s="151"/>
+      <c r="D23" s="151"/>
       <c r="E23" s="59"/>
       <c r="F23" s="28"/>
       <c r="J23" s="29"/>
@@ -52742,9 +52740,9 @@
       <c r="Y23" s="29"/>
     </row>
     <row r="24" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="148"/>
-      <c r="C24" s="145"/>
-      <c r="D24" s="145"/>
+      <c r="B24" s="156"/>
+      <c r="C24" s="151"/>
+      <c r="D24" s="151"/>
       <c r="E24" s="59"/>
       <c r="F24" s="35"/>
       <c r="G24" s="61"/>
@@ -52758,9 +52756,9 @@
       <c r="Y24" s="29"/>
     </row>
     <row r="25" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="148"/>
-      <c r="C25" s="145"/>
-      <c r="D25" s="145"/>
+      <c r="B25" s="156"/>
+      <c r="C25" s="151"/>
+      <c r="D25" s="151"/>
       <c r="E25" s="59"/>
       <c r="F25" s="28"/>
       <c r="J25" s="29"/>
@@ -52776,9 +52774,9 @@
       <c r="Y25" s="34"/>
     </row>
     <row r="26" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="148"/>
-      <c r="C26" s="145"/>
-      <c r="D26" s="145"/>
+      <c r="B26" s="156"/>
+      <c r="C26" s="151"/>
+      <c r="D26" s="151"/>
       <c r="E26" s="59"/>
       <c r="F26" s="28"/>
       <c r="J26" s="29"/>
@@ -52794,9 +52792,9 @@
       <c r="Y26" s="34"/>
     </row>
     <row r="27" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="149"/>
-      <c r="C27" s="146"/>
-      <c r="D27" s="146"/>
+      <c r="B27" s="157"/>
+      <c r="C27" s="162"/>
+      <c r="D27" s="162"/>
       <c r="E27" s="77"/>
       <c r="F27" s="30"/>
       <c r="G27" s="31"/>
@@ -52829,43 +52827,43 @@
       <c r="Y28" s="29"/>
     </row>
     <row r="29" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="150" t="s">
+      <c r="B29" s="176" t="s">
         <v>734</v>
       </c>
-      <c r="C29" s="151" t="s">
+      <c r="C29" s="158" t="s">
         <v>40</v>
       </c>
-      <c r="D29" s="173" t="s">
+      <c r="D29" s="161" t="s">
         <v>729</v>
       </c>
       <c r="E29" s="75"/>
-      <c r="F29" s="137" t="s">
+      <c r="F29" s="168" t="s">
         <v>736</v>
       </c>
-      <c r="G29" s="132"/>
-      <c r="H29" s="133"/>
-      <c r="I29" s="133"/>
-      <c r="J29" s="134"/>
-      <c r="K29" s="131"/>
-      <c r="L29" s="132"/>
-      <c r="M29" s="133"/>
-      <c r="N29" s="133"/>
-      <c r="O29" s="134"/>
-      <c r="P29" s="131"/>
-      <c r="Q29" s="132"/>
-      <c r="R29" s="133"/>
-      <c r="S29" s="133"/>
-      <c r="T29" s="134"/>
-      <c r="U29" s="135"/>
-      <c r="V29" s="136"/>
-      <c r="W29" s="133"/>
-      <c r="X29" s="133"/>
-      <c r="Y29" s="134"/>
+      <c r="G29" s="165"/>
+      <c r="H29" s="166"/>
+      <c r="I29" s="166"/>
+      <c r="J29" s="167"/>
+      <c r="K29" s="169"/>
+      <c r="L29" s="165"/>
+      <c r="M29" s="166"/>
+      <c r="N29" s="166"/>
+      <c r="O29" s="167"/>
+      <c r="P29" s="169"/>
+      <c r="Q29" s="165"/>
+      <c r="R29" s="166"/>
+      <c r="S29" s="166"/>
+      <c r="T29" s="167"/>
+      <c r="U29" s="170"/>
+      <c r="V29" s="171"/>
+      <c r="W29" s="166"/>
+      <c r="X29" s="166"/>
+      <c r="Y29" s="167"/>
     </row>
     <row r="30" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B30" s="148"/>
-      <c r="C30" s="152"/>
-      <c r="D30" s="145"/>
+      <c r="B30" s="156"/>
+      <c r="C30" s="159"/>
+      <c r="D30" s="151"/>
       <c r="E30" s="76"/>
       <c r="F30" s="26" t="s">
         <v>46</v>
@@ -52929,9 +52927,9 @@
       </c>
     </row>
     <row r="31" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="148"/>
-      <c r="C31" s="152"/>
-      <c r="D31" s="145"/>
+      <c r="B31" s="156"/>
+      <c r="C31" s="159"/>
+      <c r="D31" s="151"/>
       <c r="E31" s="67" t="s">
         <v>43</v>
       </c>
@@ -52954,9 +52952,9 @@
       <c r="Y31" s="29"/>
     </row>
     <row r="32" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="148"/>
-      <c r="C32" s="152"/>
-      <c r="D32" s="145"/>
+      <c r="B32" s="156"/>
+      <c r="C32" s="159"/>
+      <c r="D32" s="151"/>
       <c r="E32" s="60"/>
       <c r="F32" s="33"/>
       <c r="G32" s="66"/>
@@ -52971,9 +52969,9 @@
       <c r="Y32" s="29"/>
     </row>
     <row r="33" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="148"/>
-      <c r="C33" s="153"/>
-      <c r="D33" s="146"/>
+      <c r="B33" s="156"/>
+      <c r="C33" s="160"/>
+      <c r="D33" s="162"/>
       <c r="E33" s="79"/>
       <c r="F33" s="30"/>
       <c r="G33" s="31"/>
@@ -52997,43 +52995,43 @@
       <c r="Y33" s="32"/>
     </row>
     <row r="34" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="148"/>
-      <c r="C34" s="151" t="s">
+      <c r="B34" s="156"/>
+      <c r="C34" s="158" t="s">
         <v>41</v>
       </c>
-      <c r="D34" s="173" t="s">
+      <c r="D34" s="161" t="s">
         <v>730</v>
       </c>
       <c r="E34" s="75"/>
-      <c r="F34" s="137" t="s">
+      <c r="F34" s="168" t="s">
         <v>737</v>
       </c>
-      <c r="G34" s="132"/>
-      <c r="H34" s="133"/>
-      <c r="I34" s="133"/>
-      <c r="J34" s="134"/>
-      <c r="K34" s="137" t="s">
+      <c r="G34" s="165"/>
+      <c r="H34" s="166"/>
+      <c r="I34" s="166"/>
+      <c r="J34" s="167"/>
+      <c r="K34" s="168" t="s">
         <v>728</v>
       </c>
-      <c r="L34" s="136"/>
-      <c r="M34" s="133"/>
-      <c r="N34" s="133"/>
-      <c r="O34" s="134"/>
-      <c r="P34" s="131"/>
-      <c r="Q34" s="132"/>
-      <c r="R34" s="133"/>
-      <c r="S34" s="133"/>
-      <c r="T34" s="134"/>
-      <c r="U34" s="135"/>
-      <c r="V34" s="136"/>
-      <c r="W34" s="133"/>
-      <c r="X34" s="133"/>
-      <c r="Y34" s="134"/>
+      <c r="L34" s="171"/>
+      <c r="M34" s="166"/>
+      <c r="N34" s="166"/>
+      <c r="O34" s="167"/>
+      <c r="P34" s="169"/>
+      <c r="Q34" s="165"/>
+      <c r="R34" s="166"/>
+      <c r="S34" s="166"/>
+      <c r="T34" s="167"/>
+      <c r="U34" s="170"/>
+      <c r="V34" s="171"/>
+      <c r="W34" s="166"/>
+      <c r="X34" s="166"/>
+      <c r="Y34" s="167"/>
     </row>
     <row r="35" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B35" s="148"/>
-      <c r="C35" s="152"/>
-      <c r="D35" s="145"/>
+      <c r="B35" s="156"/>
+      <c r="C35" s="159"/>
+      <c r="D35" s="151"/>
       <c r="E35" s="76"/>
       <c r="F35" s="26" t="s">
         <v>46</v>
@@ -53077,9 +53075,9 @@
       <c r="Y35" s="27"/>
     </row>
     <row r="36" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B36" s="148"/>
-      <c r="C36" s="152"/>
-      <c r="D36" s="145"/>
+      <c r="B36" s="156"/>
+      <c r="C36" s="159"/>
+      <c r="D36" s="151"/>
       <c r="E36" s="67" t="s">
         <v>731</v>
       </c>
@@ -53101,9 +53099,9 @@
       <c r="Y36" s="29"/>
     </row>
     <row r="37" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B37" s="148"/>
-      <c r="C37" s="152"/>
-      <c r="D37" s="145"/>
+      <c r="B37" s="156"/>
+      <c r="C37" s="159"/>
+      <c r="D37" s="151"/>
       <c r="E37" s="59"/>
       <c r="F37" s="28"/>
       <c r="J37" s="29"/>
@@ -53115,9 +53113,9 @@
       <c r="Y37" s="29"/>
     </row>
     <row r="38" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="149"/>
-      <c r="C38" s="153"/>
-      <c r="D38" s="146"/>
+      <c r="B38" s="157"/>
+      <c r="C38" s="160"/>
+      <c r="D38" s="162"/>
       <c r="E38" s="77"/>
       <c r="F38" s="30"/>
       <c r="G38" s="31"/>
@@ -53150,43 +53148,43 @@
       <c r="Y39" s="29"/>
     </row>
     <row r="40" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="147" t="s">
+      <c r="B40" s="155" t="s">
         <v>723</v>
       </c>
-      <c r="C40" s="151" t="s">
+      <c r="C40" s="158" t="s">
         <v>40</v>
       </c>
-      <c r="D40" s="173" t="s">
+      <c r="D40" s="161" t="s">
         <v>87</v>
       </c>
       <c r="E40" s="75"/>
-      <c r="F40" s="137" t="s">
+      <c r="F40" s="168" t="s">
         <v>738</v>
       </c>
-      <c r="G40" s="132"/>
-      <c r="H40" s="133"/>
-      <c r="I40" s="133"/>
-      <c r="J40" s="134"/>
-      <c r="K40" s="131"/>
-      <c r="L40" s="132"/>
-      <c r="M40" s="133"/>
-      <c r="N40" s="133"/>
-      <c r="O40" s="134"/>
-      <c r="P40" s="131"/>
-      <c r="Q40" s="132"/>
-      <c r="R40" s="133"/>
-      <c r="S40" s="133"/>
-      <c r="T40" s="134"/>
-      <c r="U40" s="135"/>
-      <c r="V40" s="136"/>
-      <c r="W40" s="133"/>
-      <c r="X40" s="133"/>
-      <c r="Y40" s="134"/>
+      <c r="G40" s="165"/>
+      <c r="H40" s="166"/>
+      <c r="I40" s="166"/>
+      <c r="J40" s="167"/>
+      <c r="K40" s="169"/>
+      <c r="L40" s="165"/>
+      <c r="M40" s="166"/>
+      <c r="N40" s="166"/>
+      <c r="O40" s="167"/>
+      <c r="P40" s="169"/>
+      <c r="Q40" s="165"/>
+      <c r="R40" s="166"/>
+      <c r="S40" s="166"/>
+      <c r="T40" s="167"/>
+      <c r="U40" s="170"/>
+      <c r="V40" s="171"/>
+      <c r="W40" s="166"/>
+      <c r="X40" s="166"/>
+      <c r="Y40" s="167"/>
     </row>
     <row r="41" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B41" s="148"/>
-      <c r="C41" s="152"/>
-      <c r="D41" s="145"/>
+      <c r="B41" s="156"/>
+      <c r="C41" s="159"/>
+      <c r="D41" s="151"/>
       <c r="E41" s="76"/>
       <c r="F41" s="26" t="s">
         <v>46</v>
@@ -53250,9 +53248,9 @@
       </c>
     </row>
     <row r="42" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B42" s="148"/>
-      <c r="C42" s="152"/>
-      <c r="D42" s="145"/>
+      <c r="B42" s="156"/>
+      <c r="C42" s="159"/>
+      <c r="D42" s="151"/>
       <c r="E42" s="60"/>
       <c r="F42" s="26"/>
       <c r="G42" s="6"/>
@@ -53267,9 +53265,9 @@
       <c r="Y42" s="29"/>
     </row>
     <row r="43" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B43" s="148"/>
-      <c r="C43" s="152"/>
-      <c r="D43" s="145"/>
+      <c r="B43" s="156"/>
+      <c r="C43" s="159"/>
+      <c r="D43" s="151"/>
       <c r="E43" s="76"/>
       <c r="F43" s="26"/>
       <c r="G43" s="6"/>
@@ -53284,9 +53282,9 @@
       <c r="Y43" s="29"/>
     </row>
     <row r="44" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B44" s="148"/>
-      <c r="C44" s="152"/>
-      <c r="D44" s="145"/>
+      <c r="B44" s="156"/>
+      <c r="C44" s="159"/>
+      <c r="D44" s="151"/>
       <c r="E44" s="60"/>
       <c r="F44" s="33"/>
       <c r="G44" s="66"/>
@@ -53301,9 +53299,9 @@
       <c r="Y44" s="29"/>
     </row>
     <row r="45" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="148"/>
-      <c r="C45" s="153"/>
-      <c r="D45" s="146"/>
+      <c r="B45" s="156"/>
+      <c r="C45" s="160"/>
+      <c r="D45" s="162"/>
       <c r="E45" s="79"/>
       <c r="F45" s="30"/>
       <c r="G45" s="31"/>
@@ -53327,39 +53325,39 @@
       <c r="Y45" s="32"/>
     </row>
     <row r="46" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="148"/>
-      <c r="C46" s="151" t="s">
+      <c r="B46" s="156"/>
+      <c r="C46" s="158" t="s">
         <v>41</v>
       </c>
-      <c r="D46" s="173" t="s">
+      <c r="D46" s="161" t="s">
         <v>735</v>
       </c>
       <c r="E46" s="75"/>
-      <c r="F46" s="131"/>
-      <c r="G46" s="132"/>
-      <c r="H46" s="133"/>
-      <c r="I46" s="133"/>
-      <c r="J46" s="134"/>
-      <c r="K46" s="135"/>
-      <c r="L46" s="136"/>
-      <c r="M46" s="133"/>
-      <c r="N46" s="133"/>
-      <c r="O46" s="134"/>
-      <c r="P46" s="131"/>
-      <c r="Q46" s="132"/>
-      <c r="R46" s="133"/>
-      <c r="S46" s="133"/>
-      <c r="T46" s="134"/>
-      <c r="U46" s="135"/>
-      <c r="V46" s="136"/>
-      <c r="W46" s="133"/>
-      <c r="X46" s="133"/>
-      <c r="Y46" s="134"/>
+      <c r="F46" s="169"/>
+      <c r="G46" s="165"/>
+      <c r="H46" s="166"/>
+      <c r="I46" s="166"/>
+      <c r="J46" s="167"/>
+      <c r="K46" s="170"/>
+      <c r="L46" s="171"/>
+      <c r="M46" s="166"/>
+      <c r="N46" s="166"/>
+      <c r="O46" s="167"/>
+      <c r="P46" s="169"/>
+      <c r="Q46" s="165"/>
+      <c r="R46" s="166"/>
+      <c r="S46" s="166"/>
+      <c r="T46" s="167"/>
+      <c r="U46" s="170"/>
+      <c r="V46" s="171"/>
+      <c r="W46" s="166"/>
+      <c r="X46" s="166"/>
+      <c r="Y46" s="167"/>
     </row>
     <row r="47" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B47" s="148"/>
-      <c r="C47" s="152"/>
-      <c r="D47" s="145"/>
+      <c r="B47" s="156"/>
+      <c r="C47" s="159"/>
+      <c r="D47" s="151"/>
       <c r="E47" s="76"/>
       <c r="F47" s="26" t="s">
         <v>46</v>
@@ -53403,9 +53401,9 @@
       <c r="Y47" s="27"/>
     </row>
     <row r="48" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B48" s="148"/>
-      <c r="C48" s="152"/>
-      <c r="D48" s="145"/>
+      <c r="B48" s="156"/>
+      <c r="C48" s="159"/>
+      <c r="D48" s="151"/>
       <c r="E48" s="58"/>
       <c r="F48" s="28"/>
       <c r="J48" s="29"/>
@@ -53417,9 +53415,9 @@
       <c r="Y48" s="29"/>
     </row>
     <row r="49" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B49" s="148"/>
-      <c r="C49" s="152"/>
-      <c r="D49" s="145"/>
+      <c r="B49" s="156"/>
+      <c r="C49" s="159"/>
+      <c r="D49" s="151"/>
       <c r="E49" s="59"/>
       <c r="F49" s="28"/>
       <c r="J49" s="29"/>
@@ -53431,9 +53429,9 @@
       <c r="Y49" s="29"/>
     </row>
     <row r="50" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B50" s="148"/>
-      <c r="C50" s="152"/>
-      <c r="D50" s="145"/>
+      <c r="B50" s="156"/>
+      <c r="C50" s="159"/>
+      <c r="D50" s="151"/>
       <c r="E50" s="59"/>
       <c r="F50" s="28"/>
       <c r="J50" s="29"/>
@@ -53449,9 +53447,9 @@
       <c r="Y50" s="34"/>
     </row>
     <row r="51" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B51" s="148"/>
-      <c r="C51" s="152"/>
-      <c r="D51" s="145"/>
+      <c r="B51" s="156"/>
+      <c r="C51" s="159"/>
+      <c r="D51" s="151"/>
       <c r="E51" s="59"/>
       <c r="F51" s="28"/>
       <c r="J51" s="29"/>
@@ -53467,9 +53465,9 @@
       <c r="Y51" s="34"/>
     </row>
     <row r="52" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="149"/>
-      <c r="C52" s="153"/>
-      <c r="D52" s="146"/>
+      <c r="B52" s="157"/>
+      <c r="C52" s="160"/>
+      <c r="D52" s="162"/>
       <c r="E52" s="77"/>
       <c r="F52" s="30"/>
       <c r="G52" s="31"/>
@@ -53494,76 +53492,76 @@
     </row>
     <row r="53" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="54" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="140" t="s">
+      <c r="B54" s="172" t="s">
         <v>567</v>
       </c>
-      <c r="C54" s="141"/>
-      <c r="D54" s="141"/>
-      <c r="E54" s="142"/>
-      <c r="F54" s="142"/>
-      <c r="G54" s="142"/>
-      <c r="H54" s="142"/>
-      <c r="I54" s="142"/>
-      <c r="J54" s="142"/>
-      <c r="K54" s="142"/>
-      <c r="L54" s="142"/>
-      <c r="M54" s="142"/>
-      <c r="N54" s="142"/>
-      <c r="O54" s="142"/>
-      <c r="P54" s="142"/>
-      <c r="Q54" s="142"/>
-      <c r="R54" s="142"/>
-      <c r="S54" s="142"/>
-      <c r="T54" s="142"/>
-      <c r="U54" s="142"/>
-      <c r="V54" s="142"/>
-      <c r="W54" s="142"/>
-      <c r="X54" s="142"/>
-      <c r="Y54" s="143"/>
+      <c r="C54" s="173"/>
+      <c r="D54" s="173"/>
+      <c r="E54" s="174"/>
+      <c r="F54" s="174"/>
+      <c r="G54" s="174"/>
+      <c r="H54" s="174"/>
+      <c r="I54" s="174"/>
+      <c r="J54" s="174"/>
+      <c r="K54" s="174"/>
+      <c r="L54" s="174"/>
+      <c r="M54" s="174"/>
+      <c r="N54" s="174"/>
+      <c r="O54" s="174"/>
+      <c r="P54" s="174"/>
+      <c r="Q54" s="174"/>
+      <c r="R54" s="174"/>
+      <c r="S54" s="174"/>
+      <c r="T54" s="174"/>
+      <c r="U54" s="174"/>
+      <c r="V54" s="174"/>
+      <c r="W54" s="174"/>
+      <c r="X54" s="174"/>
+      <c r="Y54" s="175"/>
     </row>
     <row r="55" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="160" t="str">
+      <c r="B55" s="152" t="str">
         <f>B3</f>
         <v>RainPoint 4</v>
       </c>
-      <c r="C55" s="172" t="str">
+      <c r="C55" s="147" t="str">
         <f>C3</f>
         <v>Zone 1 og 2</v>
       </c>
-      <c r="D55" s="172" t="str">
+      <c r="D55" s="147" t="str">
         <f>D3</f>
         <v>Oppside</v>
       </c>
       <c r="E55" s="89"/>
-      <c r="F55" s="155" t="s">
+      <c r="F55" s="142" t="s">
         <v>559</v>
       </c>
-      <c r="G55" s="155"/>
-      <c r="H55" s="156"/>
-      <c r="I55" s="156"/>
-      <c r="J55" s="157"/>
-      <c r="K55" s="154" t="s">
+      <c r="G55" s="142"/>
+      <c r="H55" s="133"/>
+      <c r="I55" s="133"/>
+      <c r="J55" s="134"/>
+      <c r="K55" s="141" t="s">
         <v>560</v>
       </c>
-      <c r="L55" s="155"/>
-      <c r="M55" s="156"/>
-      <c r="N55" s="156"/>
-      <c r="O55" s="157"/>
-      <c r="P55" s="154"/>
-      <c r="Q55" s="155"/>
-      <c r="R55" s="156"/>
-      <c r="S55" s="156"/>
-      <c r="T55" s="157"/>
-      <c r="U55" s="158"/>
-      <c r="V55" s="159"/>
-      <c r="W55" s="156"/>
-      <c r="X55" s="156"/>
-      <c r="Y55" s="157"/>
+      <c r="L55" s="142"/>
+      <c r="M55" s="133"/>
+      <c r="N55" s="133"/>
+      <c r="O55" s="134"/>
+      <c r="P55" s="141"/>
+      <c r="Q55" s="142"/>
+      <c r="R55" s="133"/>
+      <c r="S55" s="133"/>
+      <c r="T55" s="134"/>
+      <c r="U55" s="131"/>
+      <c r="V55" s="132"/>
+      <c r="W55" s="133"/>
+      <c r="X55" s="133"/>
+      <c r="Y55" s="134"/>
     </row>
     <row r="56" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B56" s="161"/>
-      <c r="C56" s="168"/>
-      <c r="D56" s="168"/>
+      <c r="B56" s="153"/>
+      <c r="C56" s="139"/>
+      <c r="D56" s="139"/>
       <c r="E56" s="90"/>
       <c r="F56" s="91" t="s">
         <v>46</v>
@@ -53627,9 +53625,9 @@
       </c>
     </row>
     <row r="57" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B57" s="161"/>
-      <c r="C57" s="168"/>
-      <c r="D57" s="168"/>
+      <c r="B57" s="153"/>
+      <c r="C57" s="139"/>
+      <c r="D57" s="139"/>
       <c r="E57" s="95" t="str">
         <f>IF(E5="","",TEXT(TIME(VALUE(LEFT(E5,2)),VALUE(MID(E5,3,2)),0)+$C$107/24,"ttmm")&amp;" - "&amp;TEXT(TIME(VALUE(MID(E5,8,2)),VALUE(RIGHT(E5,2)),0)+$C$107/24,"ttmm"))</f>
         <v>1800 - 1830</v>
@@ -53716,9 +53714,9 @@
       </c>
     </row>
     <row r="58" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B58" s="161"/>
-      <c r="C58" s="168"/>
-      <c r="D58" s="168"/>
+      <c r="B58" s="153"/>
+      <c r="C58" s="139"/>
+      <c r="D58" s="139"/>
       <c r="E58" s="95" t="str">
         <f t="shared" ref="E58:F64" si="4">IF(E6="","",TEXT(TIME(VALUE(LEFT(E6,2)),VALUE(MID(E6,3,2)),0)+$C$107/24,"ttmm")&amp;" - "&amp;TEXT(TIME(VALUE(MID(E6,8,2)),VALUE(RIGHT(E6,2)),0)+$C$107/24,"ttmm"))</f>
         <v>1930 - 1949</v>
@@ -53805,9 +53803,9 @@
       </c>
     </row>
     <row r="59" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B59" s="161"/>
-      <c r="C59" s="168"/>
-      <c r="D59" s="168"/>
+      <c r="B59" s="153"/>
+      <c r="C59" s="139"/>
+      <c r="D59" s="139"/>
       <c r="E59" s="95" t="str">
         <f t="shared" si="4"/>
         <v>1950 - 1959</v>
@@ -53894,9 +53892,9 @@
       </c>
     </row>
     <row r="60" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B60" s="161"/>
-      <c r="C60" s="168"/>
-      <c r="D60" s="168"/>
+      <c r="B60" s="153"/>
+      <c r="C60" s="139"/>
+      <c r="D60" s="139"/>
       <c r="E60" s="95" t="str">
         <f t="shared" si="4"/>
         <v>2000 - 2009</v>
@@ -53983,9 +53981,9 @@
       </c>
     </row>
     <row r="61" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B61" s="161"/>
-      <c r="C61" s="168"/>
-      <c r="D61" s="168"/>
+      <c r="B61" s="153"/>
+      <c r="C61" s="139"/>
+      <c r="D61" s="139"/>
       <c r="E61" s="95" t="str">
         <f t="shared" si="4"/>
         <v>2010 - 2019</v>
@@ -54072,9 +54070,9 @@
       </c>
     </row>
     <row r="62" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B62" s="161"/>
-      <c r="C62" s="168"/>
-      <c r="D62" s="168"/>
+      <c r="B62" s="153"/>
+      <c r="C62" s="139"/>
+      <c r="D62" s="139"/>
       <c r="E62" s="95" t="str">
         <f t="shared" si="4"/>
         <v>2020 - 2029</v>
@@ -54161,9 +54159,9 @@
       </c>
     </row>
     <row r="63" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B63" s="161"/>
-      <c r="C63" s="168"/>
-      <c r="D63" s="168"/>
+      <c r="B63" s="153"/>
+      <c r="C63" s="139"/>
+      <c r="D63" s="139"/>
       <c r="E63" s="95" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -54250,9 +54248,9 @@
       </c>
     </row>
     <row r="64" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B64" s="161"/>
-      <c r="C64" s="169"/>
-      <c r="D64" s="169"/>
+      <c r="B64" s="153"/>
+      <c r="C64" s="140"/>
+      <c r="D64" s="140"/>
       <c r="E64" s="95" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -54339,45 +54337,45 @@
       </c>
     </row>
     <row r="65" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B65" s="161"/>
-      <c r="C65" s="172" t="str">
+      <c r="B65" s="153"/>
+      <c r="C65" s="147" t="str">
         <f>C13</f>
         <v>Zone 3</v>
       </c>
-      <c r="D65" s="172" t="str">
+      <c r="D65" s="147" t="str">
         <f>D13</f>
         <v>Nedside</v>
       </c>
       <c r="E65" s="89"/>
-      <c r="F65" s="155" t="s">
+      <c r="F65" s="142" t="s">
         <v>562</v>
       </c>
-      <c r="G65" s="155"/>
-      <c r="H65" s="156"/>
-      <c r="I65" s="156"/>
-      <c r="J65" s="157"/>
-      <c r="K65" s="158" t="s">
+      <c r="G65" s="142"/>
+      <c r="H65" s="133"/>
+      <c r="I65" s="133"/>
+      <c r="J65" s="134"/>
+      <c r="K65" s="131" t="s">
         <v>564</v>
       </c>
-      <c r="L65" s="159"/>
-      <c r="M65" s="156"/>
-      <c r="N65" s="156"/>
-      <c r="O65" s="157"/>
-      <c r="P65" s="154"/>
-      <c r="Q65" s="155"/>
-      <c r="R65" s="156"/>
-      <c r="S65" s="156"/>
-      <c r="T65" s="157"/>
-      <c r="U65" s="158"/>
-      <c r="V65" s="159"/>
-      <c r="W65" s="156"/>
-      <c r="X65" s="156"/>
-      <c r="Y65" s="157"/>
+      <c r="L65" s="132"/>
+      <c r="M65" s="133"/>
+      <c r="N65" s="133"/>
+      <c r="O65" s="134"/>
+      <c r="P65" s="141"/>
+      <c r="Q65" s="142"/>
+      <c r="R65" s="133"/>
+      <c r="S65" s="133"/>
+      <c r="T65" s="134"/>
+      <c r="U65" s="131"/>
+      <c r="V65" s="132"/>
+      <c r="W65" s="133"/>
+      <c r="X65" s="133"/>
+      <c r="Y65" s="134"/>
     </row>
     <row r="66" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B66" s="161"/>
-      <c r="C66" s="168"/>
-      <c r="D66" s="168"/>
+      <c r="B66" s="153"/>
+      <c r="C66" s="139"/>
+      <c r="D66" s="139"/>
       <c r="E66" s="90"/>
       <c r="F66" s="91" t="s">
         <v>46</v>
@@ -54441,9 +54439,9 @@
       </c>
     </row>
     <row r="67" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B67" s="161"/>
-      <c r="C67" s="168"/>
-      <c r="D67" s="168"/>
+      <c r="B67" s="153"/>
+      <c r="C67" s="139"/>
+      <c r="D67" s="139"/>
       <c r="E67" s="106" t="str">
         <f t="shared" ref="E67:F71" si="48">IF(E15="","",TEXT(TIME(VALUE(LEFT(E15,2)),VALUE(MID(E15,3,2)),0)+$C$107/24,"ttmm")&amp;" - "&amp;TEXT(TIME(VALUE(MID(E15,8,2)),VALUE(RIGHT(E15,2)),0)+$C$107/24,"ttmm"))</f>
         <v>2030 - 2049</v>
@@ -54530,9 +54528,9 @@
       </c>
     </row>
     <row r="68" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B68" s="161"/>
-      <c r="C68" s="168"/>
-      <c r="D68" s="168"/>
+      <c r="B68" s="153"/>
+      <c r="C68" s="139"/>
+      <c r="D68" s="139"/>
       <c r="E68" s="106" t="str">
         <f t="shared" si="48"/>
         <v>2050 - 2109</v>
@@ -54619,10 +54617,10 @@
       </c>
     </row>
     <row r="69" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B69" s="161"/>
-      <c r="C69" s="168"/>
-      <c r="D69" s="168"/>
-      <c r="E69" s="174" t="str">
+      <c r="B69" s="153"/>
+      <c r="C69" s="139"/>
+      <c r="D69" s="139"/>
+      <c r="E69" s="144" t="str">
         <f t="shared" si="48"/>
         <v>2110 - 2229</v>
       </c>
@@ -54708,10 +54706,10 @@
       </c>
     </row>
     <row r="70" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B70" s="161"/>
-      <c r="C70" s="168"/>
-      <c r="D70" s="168"/>
-      <c r="E70" s="175" t="str">
+      <c r="B70" s="153"/>
+      <c r="C70" s="139"/>
+      <c r="D70" s="139"/>
+      <c r="E70" s="145" t="str">
         <f t="shared" si="48"/>
         <v/>
       </c>
@@ -54797,10 +54795,10 @@
       </c>
     </row>
     <row r="71" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B71" s="161"/>
-      <c r="C71" s="168"/>
-      <c r="D71" s="168"/>
-      <c r="E71" s="176" t="str">
+      <c r="B71" s="153"/>
+      <c r="C71" s="139"/>
+      <c r="D71" s="139"/>
+      <c r="E71" s="146" t="str">
         <f t="shared" si="48"/>
         <v/>
       </c>
@@ -54886,43 +54884,43 @@
       </c>
     </row>
     <row r="72" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B72" s="161"/>
-      <c r="C72" s="172" t="str">
+      <c r="B72" s="153"/>
+      <c r="C72" s="147" t="str">
         <f>C20</f>
         <v>Zone 4</v>
       </c>
-      <c r="D72" s="167" t="str">
+      <c r="D72" s="138" t="str">
         <f>D20</f>
         <v>Nedside</v>
       </c>
       <c r="E72" s="108"/>
-      <c r="F72" s="170" t="s">
+      <c r="F72" s="143" t="s">
         <v>728</v>
       </c>
-      <c r="G72" s="155"/>
-      <c r="H72" s="155"/>
-      <c r="I72" s="155"/>
-      <c r="J72" s="177"/>
-      <c r="K72" s="158"/>
-      <c r="L72" s="159"/>
-      <c r="M72" s="159"/>
-      <c r="N72" s="159"/>
-      <c r="O72" s="178"/>
-      <c r="P72" s="154"/>
-      <c r="Q72" s="155"/>
-      <c r="R72" s="155"/>
-      <c r="S72" s="155"/>
-      <c r="T72" s="177"/>
-      <c r="U72" s="158"/>
-      <c r="V72" s="159"/>
-      <c r="W72" s="159"/>
-      <c r="X72" s="159"/>
-      <c r="Y72" s="178"/>
+      <c r="G72" s="142"/>
+      <c r="H72" s="142"/>
+      <c r="I72" s="142"/>
+      <c r="J72" s="148"/>
+      <c r="K72" s="131"/>
+      <c r="L72" s="132"/>
+      <c r="M72" s="132"/>
+      <c r="N72" s="132"/>
+      <c r="O72" s="149"/>
+      <c r="P72" s="141"/>
+      <c r="Q72" s="142"/>
+      <c r="R72" s="142"/>
+      <c r="S72" s="142"/>
+      <c r="T72" s="148"/>
+      <c r="U72" s="131"/>
+      <c r="V72" s="132"/>
+      <c r="W72" s="132"/>
+      <c r="X72" s="132"/>
+      <c r="Y72" s="149"/>
     </row>
     <row r="73" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B73" s="161"/>
-      <c r="C73" s="168"/>
-      <c r="D73" s="168"/>
+      <c r="B73" s="153"/>
+      <c r="C73" s="139"/>
+      <c r="D73" s="139"/>
       <c r="E73" s="109"/>
       <c r="F73" s="91" t="s">
         <v>46</v>
@@ -54986,9 +54984,9 @@
       </c>
     </row>
     <row r="74" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B74" s="161"/>
-      <c r="C74" s="168"/>
-      <c r="D74" s="168"/>
+      <c r="B74" s="153"/>
+      <c r="C74" s="139"/>
+      <c r="D74" s="139"/>
       <c r="E74" s="95" t="str">
         <f t="shared" ref="E74:F79" si="84">IF(E22="","",TEXT(TIME(VALUE(LEFT(E22,2)),VALUE(MID(E22,3,2)),0)+$C$107/24,"ttmm")&amp;" - "&amp;TEXT(TIME(VALUE(MID(E22,8,2)),VALUE(RIGHT(E22,2)),0)+$C$107/24,"ttmm"))</f>
         <v>2230 - 2233</v>
@@ -55051,9 +55049,9 @@
       <c r="Y74" s="111"/>
     </row>
     <row r="75" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B75" s="161"/>
-      <c r="C75" s="168"/>
-      <c r="D75" s="168"/>
+      <c r="B75" s="153"/>
+      <c r="C75" s="139"/>
+      <c r="D75" s="139"/>
       <c r="E75" s="112" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -55116,9 +55114,9 @@
       <c r="Y75" s="111"/>
     </row>
     <row r="76" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B76" s="161"/>
-      <c r="C76" s="168"/>
-      <c r="D76" s="168"/>
+      <c r="B76" s="153"/>
+      <c r="C76" s="139"/>
+      <c r="D76" s="139"/>
       <c r="E76" s="112" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -55181,9 +55179,9 @@
       <c r="Y76" s="111"/>
     </row>
     <row r="77" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B77" s="161"/>
-      <c r="C77" s="168"/>
-      <c r="D77" s="168"/>
+      <c r="B77" s="153"/>
+      <c r="C77" s="139"/>
+      <c r="D77" s="139"/>
       <c r="E77" s="112" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -55246,9 +55244,9 @@
       <c r="Y77" s="114"/>
     </row>
     <row r="78" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B78" s="161"/>
-      <c r="C78" s="168"/>
-      <c r="D78" s="168"/>
+      <c r="B78" s="153"/>
+      <c r="C78" s="139"/>
+      <c r="D78" s="139"/>
       <c r="E78" s="112" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -55311,9 +55309,9 @@
       <c r="Y78" s="114"/>
     </row>
     <row r="79" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B79" s="162"/>
-      <c r="C79" s="169"/>
-      <c r="D79" s="169"/>
+      <c r="B79" s="154"/>
+      <c r="C79" s="140"/>
+      <c r="D79" s="140"/>
       <c r="E79" s="115" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -55385,46 +55383,46 @@
       <c r="Y80" s="29"/>
     </row>
     <row r="81" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B81" s="163" t="str">
+      <c r="B81" s="164" t="str">
         <f>B29</f>
         <v>RainPoint 2 Home</v>
       </c>
-      <c r="C81" s="164" t="str">
+      <c r="C81" s="135" t="str">
         <f>C29</f>
         <v>Zone 1</v>
       </c>
-      <c r="D81" s="167" t="str">
+      <c r="D81" s="138" t="str">
         <f>D29</f>
         <v>Pallehus</v>
       </c>
       <c r="E81" s="108"/>
-      <c r="F81" s="170" t="s">
+      <c r="F81" s="143" t="s">
         <v>736</v>
       </c>
-      <c r="G81" s="155"/>
-      <c r="H81" s="156"/>
-      <c r="I81" s="156"/>
-      <c r="J81" s="157"/>
-      <c r="K81" s="154"/>
-      <c r="L81" s="155"/>
-      <c r="M81" s="156"/>
-      <c r="N81" s="156"/>
-      <c r="O81" s="157"/>
-      <c r="P81" s="154"/>
-      <c r="Q81" s="155"/>
-      <c r="R81" s="156"/>
-      <c r="S81" s="156"/>
-      <c r="T81" s="157"/>
-      <c r="U81" s="158"/>
-      <c r="V81" s="159"/>
-      <c r="W81" s="156"/>
-      <c r="X81" s="156"/>
-      <c r="Y81" s="157"/>
+      <c r="G81" s="142"/>
+      <c r="H81" s="133"/>
+      <c r="I81" s="133"/>
+      <c r="J81" s="134"/>
+      <c r="K81" s="141"/>
+      <c r="L81" s="142"/>
+      <c r="M81" s="133"/>
+      <c r="N81" s="133"/>
+      <c r="O81" s="134"/>
+      <c r="P81" s="141"/>
+      <c r="Q81" s="142"/>
+      <c r="R81" s="133"/>
+      <c r="S81" s="133"/>
+      <c r="T81" s="134"/>
+      <c r="U81" s="131"/>
+      <c r="V81" s="132"/>
+      <c r="W81" s="133"/>
+      <c r="X81" s="133"/>
+      <c r="Y81" s="134"/>
     </row>
     <row r="82" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B82" s="161"/>
-      <c r="C82" s="165"/>
-      <c r="D82" s="168"/>
+      <c r="B82" s="153"/>
+      <c r="C82" s="136"/>
+      <c r="D82" s="139"/>
       <c r="E82" s="109"/>
       <c r="F82" s="105" t="s">
         <v>46</v>
@@ -55488,9 +55486,9 @@
       </c>
     </row>
     <row r="83" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B83" s="161"/>
-      <c r="C83" s="165"/>
-      <c r="D83" s="168"/>
+      <c r="B83" s="153"/>
+      <c r="C83" s="136"/>
+      <c r="D83" s="139"/>
       <c r="E83" s="120" t="str">
         <f t="shared" ref="E83:F85" si="105">IF(E31="","",TEXT(TIME(VALUE(LEFT(E31,2)),VALUE(MID(E31,3,2)),0)+$C$107/24,"ttmm")&amp;" - "&amp;TEXT(TIME(VALUE(MID(E31,8,2)),VALUE(RIGHT(E31,2)),0)+$C$107/24,"ttmm"))</f>
         <v>2100 - 2102</v>
@@ -55577,9 +55575,9 @@
       </c>
     </row>
     <row r="84" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B84" s="161"/>
-      <c r="C84" s="165"/>
-      <c r="D84" s="168"/>
+      <c r="B84" s="153"/>
+      <c r="C84" s="136"/>
+      <c r="D84" s="139"/>
       <c r="E84" s="121" t="str">
         <f t="shared" si="105"/>
         <v/>
@@ -55666,9 +55664,9 @@
       </c>
     </row>
     <row r="85" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B85" s="161"/>
-      <c r="C85" s="166"/>
-      <c r="D85" s="169"/>
+      <c r="B85" s="153"/>
+      <c r="C85" s="137"/>
+      <c r="D85" s="140"/>
       <c r="E85" s="123" t="str">
         <f t="shared" si="105"/>
         <v/>
@@ -55755,45 +55753,45 @@
       </c>
     </row>
     <row r="86" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B86" s="161"/>
-      <c r="C86" s="164" t="str">
+      <c r="B86" s="153"/>
+      <c r="C86" s="135" t="str">
         <f>C34</f>
         <v>Zone 2</v>
       </c>
-      <c r="D86" s="167" t="str">
+      <c r="D86" s="138" t="str">
         <f>D34</f>
         <v>Benk</v>
       </c>
       <c r="E86" s="108"/>
-      <c r="F86" s="170" t="s">
+      <c r="F86" s="143" t="s">
         <v>737</v>
       </c>
-      <c r="G86" s="155"/>
-      <c r="H86" s="156"/>
-      <c r="I86" s="156"/>
-      <c r="J86" s="157"/>
-      <c r="K86" s="170" t="s">
+      <c r="G86" s="142"/>
+      <c r="H86" s="133"/>
+      <c r="I86" s="133"/>
+      <c r="J86" s="134"/>
+      <c r="K86" s="143" t="s">
         <v>728</v>
       </c>
-      <c r="L86" s="159"/>
-      <c r="M86" s="156"/>
-      <c r="N86" s="156"/>
-      <c r="O86" s="157"/>
-      <c r="P86" s="154"/>
-      <c r="Q86" s="155"/>
-      <c r="R86" s="156"/>
-      <c r="S86" s="156"/>
-      <c r="T86" s="157"/>
-      <c r="U86" s="158"/>
-      <c r="V86" s="159"/>
-      <c r="W86" s="156"/>
-      <c r="X86" s="156"/>
-      <c r="Y86" s="157"/>
+      <c r="L86" s="132"/>
+      <c r="M86" s="133"/>
+      <c r="N86" s="133"/>
+      <c r="O86" s="134"/>
+      <c r="P86" s="141"/>
+      <c r="Q86" s="142"/>
+      <c r="R86" s="133"/>
+      <c r="S86" s="133"/>
+      <c r="T86" s="134"/>
+      <c r="U86" s="131"/>
+      <c r="V86" s="132"/>
+      <c r="W86" s="133"/>
+      <c r="X86" s="133"/>
+      <c r="Y86" s="134"/>
     </row>
     <row r="87" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B87" s="161"/>
-      <c r="C87" s="165"/>
-      <c r="D87" s="168"/>
+      <c r="B87" s="153"/>
+      <c r="C87" s="136"/>
+      <c r="D87" s="139"/>
       <c r="E87" s="109"/>
       <c r="F87" s="91" t="s">
         <v>46</v>
@@ -55837,9 +55835,9 @@
       <c r="Y87" s="94"/>
     </row>
     <row r="88" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B88" s="161"/>
-      <c r="C88" s="165"/>
-      <c r="D88" s="168"/>
+      <c r="B88" s="153"/>
+      <c r="C88" s="136"/>
+      <c r="D88" s="139"/>
       <c r="E88" s="120" t="str">
         <f t="shared" ref="E88:F90" si="128">IF(E36="","",TEXT(TIME(VALUE(LEFT(E36,2)),VALUE(MID(E36,3,2)),0)+$C$107/24,"ttmm")&amp;" - "&amp;TEXT(TIME(VALUE(MID(E36,8,2)),VALUE(RIGHT(E36,2)),0)+$C$107/24,"ttmm"))</f>
         <v>2110 - 2115</v>
@@ -55926,9 +55924,9 @@
       </c>
     </row>
     <row r="89" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B89" s="161"/>
-      <c r="C89" s="165"/>
-      <c r="D89" s="168"/>
+      <c r="B89" s="153"/>
+      <c r="C89" s="136"/>
+      <c r="D89" s="139"/>
       <c r="E89" s="112" t="str">
         <f t="shared" si="128"/>
         <v/>
@@ -56015,9 +56013,9 @@
       </c>
     </row>
     <row r="90" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B90" s="162"/>
-      <c r="C90" s="166"/>
-      <c r="D90" s="169"/>
+      <c r="B90" s="154"/>
+      <c r="C90" s="137"/>
+      <c r="D90" s="140"/>
       <c r="E90" s="115" t="str">
         <f t="shared" si="128"/>
         <v/>
@@ -56113,46 +56111,46 @@
       <c r="Y91" s="29"/>
     </row>
     <row r="92" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B92" s="160" t="str">
+      <c r="B92" s="152" t="str">
         <f>B40</f>
         <v>RainPoint 2</v>
       </c>
-      <c r="C92" s="164" t="str">
+      <c r="C92" s="135" t="str">
         <f>C40</f>
         <v>Zone 1</v>
       </c>
-      <c r="D92" s="167" t="str">
+      <c r="D92" s="138" t="str">
         <f>D40</f>
         <v>Drivhus</v>
       </c>
       <c r="E92" s="108"/>
-      <c r="F92" s="170" t="s">
+      <c r="F92" s="143" t="s">
         <v>738</v>
       </c>
-      <c r="G92" s="155"/>
-      <c r="H92" s="156"/>
-      <c r="I92" s="156"/>
-      <c r="J92" s="157"/>
-      <c r="K92" s="154"/>
-      <c r="L92" s="155"/>
-      <c r="M92" s="156"/>
-      <c r="N92" s="156"/>
-      <c r="O92" s="157"/>
-      <c r="P92" s="154"/>
-      <c r="Q92" s="155"/>
-      <c r="R92" s="156"/>
-      <c r="S92" s="156"/>
-      <c r="T92" s="157"/>
-      <c r="U92" s="158"/>
-      <c r="V92" s="159"/>
-      <c r="W92" s="156"/>
-      <c r="X92" s="156"/>
-      <c r="Y92" s="157"/>
+      <c r="G92" s="142"/>
+      <c r="H92" s="133"/>
+      <c r="I92" s="133"/>
+      <c r="J92" s="134"/>
+      <c r="K92" s="141"/>
+      <c r="L92" s="142"/>
+      <c r="M92" s="133"/>
+      <c r="N92" s="133"/>
+      <c r="O92" s="134"/>
+      <c r="P92" s="141"/>
+      <c r="Q92" s="142"/>
+      <c r="R92" s="133"/>
+      <c r="S92" s="133"/>
+      <c r="T92" s="134"/>
+      <c r="U92" s="131"/>
+      <c r="V92" s="132"/>
+      <c r="W92" s="133"/>
+      <c r="X92" s="133"/>
+      <c r="Y92" s="134"/>
     </row>
     <row r="93" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B93" s="161"/>
-      <c r="C93" s="165"/>
-      <c r="D93" s="168"/>
+      <c r="B93" s="153"/>
+      <c r="C93" s="136"/>
+      <c r="D93" s="139"/>
       <c r="E93" s="109"/>
       <c r="F93" s="105" t="s">
         <v>46</v>
@@ -56216,9 +56214,9 @@
       </c>
     </row>
     <row r="94" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B94" s="161"/>
-      <c r="C94" s="165"/>
-      <c r="D94" s="168"/>
+      <c r="B94" s="153"/>
+      <c r="C94" s="136"/>
+      <c r="D94" s="139"/>
       <c r="E94" s="121" t="str">
         <f t="shared" ref="E94:F97" si="150">IF(E42="","",TEXT(TIME(VALUE(LEFT(E42,2)),VALUE(MID(E42,3,2)),0)+$C$107/24,"ttmm")&amp;" - "&amp;TEXT(TIME(VALUE(MID(E42,8,2)),VALUE(RIGHT(E42,2)),0)+$C$107/24,"ttmm"))</f>
         <v/>
@@ -56305,9 +56303,9 @@
       </c>
     </row>
     <row r="95" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B95" s="161"/>
-      <c r="C95" s="165"/>
-      <c r="D95" s="168"/>
+      <c r="B95" s="153"/>
+      <c r="C95" s="136"/>
+      <c r="D95" s="139"/>
       <c r="E95" s="109" t="str">
         <f t="shared" si="150"/>
         <v/>
@@ -56394,9 +56392,9 @@
       </c>
     </row>
     <row r="96" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B96" s="161"/>
-      <c r="C96" s="165"/>
-      <c r="D96" s="168"/>
+      <c r="B96" s="153"/>
+      <c r="C96" s="136"/>
+      <c r="D96" s="139"/>
       <c r="E96" s="121" t="str">
         <f t="shared" si="150"/>
         <v/>
@@ -56483,9 +56481,9 @@
       </c>
     </row>
     <row r="97" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B97" s="161"/>
-      <c r="C97" s="166"/>
-      <c r="D97" s="169"/>
+      <c r="B97" s="153"/>
+      <c r="C97" s="137"/>
+      <c r="D97" s="140"/>
       <c r="E97" s="123" t="str">
         <f t="shared" si="150"/>
         <v/>
@@ -56572,41 +56570,41 @@
       </c>
     </row>
     <row r="98" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B98" s="161"/>
-      <c r="C98" s="164" t="str">
+      <c r="B98" s="153"/>
+      <c r="C98" s="135" t="str">
         <f>C46</f>
         <v>Zone 2</v>
       </c>
-      <c r="D98" s="167" t="str">
+      <c r="D98" s="138" t="str">
         <f>D46</f>
         <v>Fremtid plen</v>
       </c>
       <c r="E98" s="108"/>
-      <c r="F98" s="154"/>
-      <c r="G98" s="155"/>
-      <c r="H98" s="156"/>
-      <c r="I98" s="156"/>
-      <c r="J98" s="157"/>
-      <c r="K98" s="158"/>
-      <c r="L98" s="159"/>
-      <c r="M98" s="156"/>
-      <c r="N98" s="156"/>
-      <c r="O98" s="157"/>
-      <c r="P98" s="154"/>
-      <c r="Q98" s="155"/>
-      <c r="R98" s="156"/>
-      <c r="S98" s="156"/>
-      <c r="T98" s="157"/>
-      <c r="U98" s="158"/>
-      <c r="V98" s="159"/>
-      <c r="W98" s="156"/>
-      <c r="X98" s="156"/>
-      <c r="Y98" s="157"/>
+      <c r="F98" s="141"/>
+      <c r="G98" s="142"/>
+      <c r="H98" s="133"/>
+      <c r="I98" s="133"/>
+      <c r="J98" s="134"/>
+      <c r="K98" s="131"/>
+      <c r="L98" s="132"/>
+      <c r="M98" s="133"/>
+      <c r="N98" s="133"/>
+      <c r="O98" s="134"/>
+      <c r="P98" s="141"/>
+      <c r="Q98" s="142"/>
+      <c r="R98" s="133"/>
+      <c r="S98" s="133"/>
+      <c r="T98" s="134"/>
+      <c r="U98" s="131"/>
+      <c r="V98" s="132"/>
+      <c r="W98" s="133"/>
+      <c r="X98" s="133"/>
+      <c r="Y98" s="134"/>
     </row>
     <row r="99" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B99" s="161"/>
-      <c r="C99" s="165"/>
-      <c r="D99" s="168"/>
+      <c r="B99" s="153"/>
+      <c r="C99" s="136"/>
+      <c r="D99" s="139"/>
       <c r="E99" s="109"/>
       <c r="F99" s="105" t="s">
         <v>46</v>
@@ -56670,9 +56668,9 @@
       </c>
     </row>
     <row r="100" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B100" s="161"/>
-      <c r="C100" s="165"/>
-      <c r="D100" s="168"/>
+      <c r="B100" s="153"/>
+      <c r="C100" s="136"/>
+      <c r="D100" s="139"/>
       <c r="E100" s="125" t="str">
         <f t="shared" ref="E100:F104" si="179">IF(E48="","",TEXT(TIME(VALUE(LEFT(E48,2)),VALUE(MID(E48,3,2)),0)+$C$107/24,"ttmm")&amp;" - "&amp;TEXT(TIME(VALUE(MID(E48,8,2)),VALUE(RIGHT(E48,2)),0)+$C$107/24,"ttmm"))</f>
         <v/>
@@ -56759,9 +56757,9 @@
       </c>
     </row>
     <row r="101" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B101" s="161"/>
-      <c r="C101" s="165"/>
-      <c r="D101" s="168"/>
+      <c r="B101" s="153"/>
+      <c r="C101" s="136"/>
+      <c r="D101" s="139"/>
       <c r="E101" s="112" t="str">
         <f t="shared" si="179"/>
         <v/>
@@ -56848,9 +56846,9 @@
       </c>
     </row>
     <row r="102" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B102" s="161"/>
-      <c r="C102" s="165"/>
-      <c r="D102" s="168"/>
+      <c r="B102" s="153"/>
+      <c r="C102" s="136"/>
+      <c r="D102" s="139"/>
       <c r="E102" s="112" t="str">
         <f t="shared" si="179"/>
         <v/>
@@ -56937,9 +56935,9 @@
       </c>
     </row>
     <row r="103" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B103" s="161"/>
-      <c r="C103" s="165"/>
-      <c r="D103" s="168"/>
+      <c r="B103" s="153"/>
+      <c r="C103" s="136"/>
+      <c r="D103" s="139"/>
       <c r="E103" s="112" t="str">
         <f t="shared" si="179"/>
         <v/>
@@ -57026,9 +57024,9 @@
       </c>
     </row>
     <row r="104" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B104" s="162"/>
-      <c r="C104" s="166"/>
-      <c r="D104" s="169"/>
+      <c r="B104" s="154"/>
+      <c r="C104" s="137"/>
+      <c r="D104" s="140"/>
       <c r="E104" s="115" t="str">
         <f t="shared" si="179"/>
         <v/>
@@ -57135,58 +57133,32 @@
     </row>
   </sheetData>
   <mergeCells count="94">
-    <mergeCell ref="U92:Y92"/>
-    <mergeCell ref="C98:C104"/>
-    <mergeCell ref="D98:D104"/>
-    <mergeCell ref="F98:J98"/>
-    <mergeCell ref="K98:O98"/>
-    <mergeCell ref="P98:T98"/>
-    <mergeCell ref="U98:Y98"/>
-    <mergeCell ref="C92:C97"/>
-    <mergeCell ref="D92:D97"/>
-    <mergeCell ref="F92:J92"/>
-    <mergeCell ref="K92:O92"/>
-    <mergeCell ref="P92:T92"/>
-    <mergeCell ref="U81:Y81"/>
-    <mergeCell ref="C86:C90"/>
-    <mergeCell ref="D86:D90"/>
-    <mergeCell ref="F86:J86"/>
-    <mergeCell ref="K86:O86"/>
-    <mergeCell ref="P86:T86"/>
-    <mergeCell ref="U86:Y86"/>
-    <mergeCell ref="U65:Y65"/>
-    <mergeCell ref="E69:E71"/>
-    <mergeCell ref="C72:C79"/>
-    <mergeCell ref="D72:D79"/>
-    <mergeCell ref="F72:J72"/>
-    <mergeCell ref="K72:O72"/>
-    <mergeCell ref="P72:T72"/>
-    <mergeCell ref="U72:Y72"/>
-    <mergeCell ref="E17:E19"/>
-    <mergeCell ref="B55:B79"/>
-    <mergeCell ref="C55:C64"/>
-    <mergeCell ref="D55:D64"/>
-    <mergeCell ref="C65:C71"/>
-    <mergeCell ref="D65:D71"/>
-    <mergeCell ref="B40:B52"/>
-    <mergeCell ref="C40:C45"/>
-    <mergeCell ref="C46:C52"/>
-    <mergeCell ref="D29:D33"/>
-    <mergeCell ref="D40:D45"/>
-    <mergeCell ref="D13:D19"/>
-    <mergeCell ref="D20:D27"/>
-    <mergeCell ref="D34:D38"/>
-    <mergeCell ref="D46:D52"/>
-    <mergeCell ref="B92:B104"/>
-    <mergeCell ref="F65:J65"/>
-    <mergeCell ref="K65:O65"/>
-    <mergeCell ref="F55:J55"/>
-    <mergeCell ref="K55:O55"/>
-    <mergeCell ref="B81:B90"/>
-    <mergeCell ref="C81:C85"/>
-    <mergeCell ref="D81:D85"/>
-    <mergeCell ref="F81:J81"/>
-    <mergeCell ref="K81:O81"/>
+    <mergeCell ref="P46:T46"/>
+    <mergeCell ref="K46:O46"/>
+    <mergeCell ref="P13:T13"/>
+    <mergeCell ref="K29:O29"/>
+    <mergeCell ref="P29:T29"/>
+    <mergeCell ref="U13:Y13"/>
+    <mergeCell ref="F20:J20"/>
+    <mergeCell ref="K20:O20"/>
+    <mergeCell ref="P20:T20"/>
+    <mergeCell ref="U20:Y20"/>
+    <mergeCell ref="B2:Y2"/>
+    <mergeCell ref="F13:J13"/>
+    <mergeCell ref="K13:O13"/>
+    <mergeCell ref="B54:Y54"/>
+    <mergeCell ref="U3:Y3"/>
+    <mergeCell ref="K3:O3"/>
+    <mergeCell ref="P3:T3"/>
+    <mergeCell ref="D3:D12"/>
+    <mergeCell ref="C3:C12"/>
+    <mergeCell ref="C13:C19"/>
+    <mergeCell ref="C20:C27"/>
+    <mergeCell ref="B3:B27"/>
+    <mergeCell ref="B29:B38"/>
+    <mergeCell ref="C29:C33"/>
+    <mergeCell ref="C34:C38"/>
+    <mergeCell ref="U29:Y29"/>
     <mergeCell ref="P55:T55"/>
     <mergeCell ref="P65:T65"/>
     <mergeCell ref="P81:T81"/>
@@ -57203,32 +57175,58 @@
     <mergeCell ref="K40:O40"/>
     <mergeCell ref="P40:T40"/>
     <mergeCell ref="U40:Y40"/>
-    <mergeCell ref="B2:Y2"/>
-    <mergeCell ref="F13:J13"/>
-    <mergeCell ref="K13:O13"/>
-    <mergeCell ref="B54:Y54"/>
-    <mergeCell ref="U3:Y3"/>
-    <mergeCell ref="K3:O3"/>
-    <mergeCell ref="P3:T3"/>
-    <mergeCell ref="D3:D12"/>
-    <mergeCell ref="C3:C12"/>
-    <mergeCell ref="C13:C19"/>
-    <mergeCell ref="C20:C27"/>
-    <mergeCell ref="B3:B27"/>
-    <mergeCell ref="B29:B38"/>
-    <mergeCell ref="C29:C33"/>
-    <mergeCell ref="C34:C38"/>
-    <mergeCell ref="U29:Y29"/>
-    <mergeCell ref="U13:Y13"/>
-    <mergeCell ref="F20:J20"/>
-    <mergeCell ref="K20:O20"/>
-    <mergeCell ref="P20:T20"/>
-    <mergeCell ref="U20:Y20"/>
-    <mergeCell ref="P46:T46"/>
-    <mergeCell ref="K46:O46"/>
-    <mergeCell ref="P13:T13"/>
-    <mergeCell ref="K29:O29"/>
-    <mergeCell ref="P29:T29"/>
+    <mergeCell ref="B92:B104"/>
+    <mergeCell ref="F65:J65"/>
+    <mergeCell ref="K65:O65"/>
+    <mergeCell ref="F55:J55"/>
+    <mergeCell ref="K55:O55"/>
+    <mergeCell ref="B81:B90"/>
+    <mergeCell ref="C81:C85"/>
+    <mergeCell ref="D81:D85"/>
+    <mergeCell ref="F81:J81"/>
+    <mergeCell ref="K81:O81"/>
+    <mergeCell ref="E17:E19"/>
+    <mergeCell ref="B55:B79"/>
+    <mergeCell ref="C55:C64"/>
+    <mergeCell ref="D55:D64"/>
+    <mergeCell ref="C65:C71"/>
+    <mergeCell ref="D65:D71"/>
+    <mergeCell ref="B40:B52"/>
+    <mergeCell ref="C40:C45"/>
+    <mergeCell ref="C46:C52"/>
+    <mergeCell ref="D29:D33"/>
+    <mergeCell ref="D40:D45"/>
+    <mergeCell ref="D13:D19"/>
+    <mergeCell ref="D20:D27"/>
+    <mergeCell ref="D34:D38"/>
+    <mergeCell ref="D46:D52"/>
+    <mergeCell ref="U65:Y65"/>
+    <mergeCell ref="E69:E71"/>
+    <mergeCell ref="C72:C79"/>
+    <mergeCell ref="D72:D79"/>
+    <mergeCell ref="F72:J72"/>
+    <mergeCell ref="K72:O72"/>
+    <mergeCell ref="P72:T72"/>
+    <mergeCell ref="U72:Y72"/>
+    <mergeCell ref="U81:Y81"/>
+    <mergeCell ref="C86:C90"/>
+    <mergeCell ref="D86:D90"/>
+    <mergeCell ref="F86:J86"/>
+    <mergeCell ref="K86:O86"/>
+    <mergeCell ref="P86:T86"/>
+    <mergeCell ref="U86:Y86"/>
+    <mergeCell ref="U92:Y92"/>
+    <mergeCell ref="C98:C104"/>
+    <mergeCell ref="D98:D104"/>
+    <mergeCell ref="F98:J98"/>
+    <mergeCell ref="K98:O98"/>
+    <mergeCell ref="P98:T98"/>
+    <mergeCell ref="U98:Y98"/>
+    <mergeCell ref="C92:C97"/>
+    <mergeCell ref="D92:D97"/>
+    <mergeCell ref="F92:J92"/>
+    <mergeCell ref="K92:O92"/>
+    <mergeCell ref="P92:T92"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="60" orientation="landscape" verticalDpi="0" r:id="rId1"/>
@@ -57242,17 +57240,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D06CFA42-8E17-446B-A60F-405E706C4F43}">
   <dimension ref="A2:K25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.76171875" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.23828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.9140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.8359375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.9140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.9296875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="31" customWidth="1"/>
+    <col min="10" max="10" width="18.0234375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="30.9375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">

</xml_diff>